<commit_message>
tracker: A4 done + A2/A4 work-log rows
Regenerate Docs/Prasad_TrackA_Task_Tracker.xlsx (via build_prasad_tracker.py):
A4 Ingestion API -> in progress with detail, A6 marked next, and Work Log rows
for A2 (d8fc10b) and A4 (ee06657).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgpcHPiZiSoedUk6eogriY
</commit_message>
<xml_diff>
--- a/Docs/Prasad_TrackA_Task_Tracker.xlsx
+++ b/Docs/Prasad_TrackA_Task_Tracker.xlsx
@@ -841,7 +841,7 @@
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>NEXT (with A4). Build before A5 — the Trigger Engine depends on it. Depends on A2. reference.would_fire is the executable spec to delegate to.</t>
+          <t>NEXT. Build before A5 — the Trigger Engine depends on it. Depends on A2. reference.would_fire is the executable spec to delegate to.</t>
         </is>
       </c>
     </row>
@@ -866,17 +866,25 @@
           <t>Track A</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Core done + tested. The single write-door in services/event_pipeline/ingestion/: POST /v1/events + POST /v1/events:batch (partial-success) writing through A2's transactional outbox. Single-event body IS generator.models.Event, so FastAPI validation + extra='forbid' is the PII field allow-list (POA/15 §4) — unknown/PII field -&gt; 422. Auth, identity binding and rate limiting sit behind seams because §10 is open: ApiKeyAuthenticator now (mTLS/JWT later; JWT would set Principal.customer_id so identity binding becomes a real cross-check), in-memory fixed-window rate limiter (Redis in prod). Idempotency delegated to the store (retry -&gt; 202 duplicate, never a second row). Outcome-&gt;status 202/409/429/503/422. build_app wires it when a store is present + accepts an injected store for tests. Deferred (POA/02 §11): real auth mechanism, distributed rate limiter, load verification.</t>
+        </is>
+      </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Depends on A2. Consumes the Event contract from generator/models.py (extra='forbid' makes malformed-event rejection testable).</t>
+          <t>services/event_pipeline/ingestion/{router,service,auth,ratelimit,schemas}.py, main.py, services/platform/config.py, pyproject (ruff), POA/02 §11; tests/test_ingestion_api.py (11, incl. e2e API-&gt;store-&gt;relay-&gt;stream) — 123 total green, ruff clean. Commit ee06657 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1435,6 +1443,33 @@
       <c r="E10" s="4" t="inlineStr">
         <is>
           <t>d8fc10b (PR #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Built the Ingestion API — the single write-door — on the A1 template, writing through A2's outbox (so no direct dual write). Kept the same discipline: the body IS the Event contract, so validation + extra='forbid' doubles as the PII field allow-list, and idempotency is the store's not a second mechanism. The §10 open questions (auth mechanism, identity token vs body, volume) are handled behind seams — API-key auth, identity binding, in-memory rate limiter — the way Shagun handled B4/B5's open transport, so none of them block code. Batch endpoint does per-item validation for partial success. Added an injected-store path to build_app for tests and an end-to-end test proving API-&gt;store-&gt;outbox-&gt;relay-&gt;stream.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>11 new tests, 123 total green; ruff clean</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>ee06657 (PR #1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: A6 done + work-log row; A5 marked next
Regenerate Docs/Prasad_TrackA_Task_Tracker.xlsx: A6 Frequency/Precedence ->
in progress with detail (commit 7a5a0f8), A5 Trigger Eval marked next, and a
Work Log row for A6.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgpcHPiZiSoedUk6eogriY
</commit_message>
<xml_diff>
--- a/Docs/Prasad_TrackA_Task_Tracker.xlsx
+++ b/Docs/Prasad_TrackA_Task_Tracker.xlsx
@@ -831,17 +831,25 @@
           <t>Track A</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Core done + tested. services/event_pipeline/frequency/: Postgres engagement ledger (source of truth; only reserved/confirmed count, rolled_back ignored), sliding-window caps that DELEGATE to reference.would_fire (so the service and the invariant suite test the same rule), per-customer global cap + ISO-8601 cooldown, deterministic precedence (weight -&gt; match specificity -&gt; most-recent signal -&gt; lowest id, order-independent), atomic reserve under a per-customer lock (concurrency test: 10 threads, cap 1 -&gt; exactly 1 fires). reserve-&gt;confirm/rollback so a failed M08 send frees the slot instead of burning the cap. Every suppression carries a reason + per-trigger losers for M14. CROSS-TRACK: A6-&gt;M08 contract (MatchCandidate/EngagementDecision/SuppressionReason) added to generator/models.py — reconcile with Shagun's local §5 handshake. Deferred (POA/05 §11): Redis counters, reservation-TTL sweep, M13 cap config. No HTTP surface (library called by A5).</t>
+        </is>
+      </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>NEXT. Build before A5 — the Trigger Engine depends on it. Depends on A2. reference.would_fire is the executable spec to delegate to.</t>
+          <t>services/event_pipeline/frequency/{tables,ledger,engine,precedence,lock,bootstrap}.py, generator/models.py (contract), POA/05 §11; tests/test_frequency_precedence.py (11) — 134 total green, ruff clean. Commit 7a5a0f8 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -919,7 +927,7 @@
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Depends on A2, A6. Code against generator/fixtures.py trigger/config defaults until B1 ships persistence. 'Fire' decision -&gt; conversation start is a Pydantic message, not a call (§5).</t>
+          <t>NEXT. Depends on A2, A6 (both done). Consumes the Redis stream (events:in / group trigger-eval), matches triggers, hands MatchCandidates to A6's reserve(), and emits the 'fire' decision as a Pydantic message (§5). Code against generator/fixtures.py trigger defaults until B1 ships persistence.</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1470,6 +1478,33 @@
       <c r="E11" s="4" t="inlineStr">
         <is>
           <t>ee06657 (PR #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Built the Frequency Cap &amp; Precedence engine — the gate A5 calls before firing. Same delegate-to-the-spec discipline as A2/A4: cap accounting hands ledger timestamps to reference.would_fire, the exact sliding-window rule test_invariants already asserts, so the service can't quietly diverge from the spec. Precedence is deterministic and order-independent (weight -&gt; specificity -&gt; recency -&gt; id). The judgement call was the reserve-&gt;confirm/rollback handshake: a reserved slot is only finalised when M08 delivers, and rolled back on failure, so a failed send doesn't burn a customer's cap — the cross-track contract I put in generator/models.py to reconcile with Shagun's local §5. Wrote the concurrency invariant test POA/05 §6 asks for (10 threads, cap 1 -&gt; exactly one fires) using a per-customer lock seam.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>11 new tests, 134 total green; ruff clean</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>7a5a0f8 (PR #1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: A5 done + work-log row; A7 marked next
Regenerate Docs/Prasad_TrackA_Task_Tracker.xlsx: A5 Trigger Evaluation ->
in progress with detail (commit 2b46310), A7 Pending Queue marked next, Work Log
row for A5.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgpcHPiZiSoedUk6eogriY
</commit_message>
<xml_diff>
--- a/Docs/Prasad_TrackA_Task_Tracker.xlsx
+++ b/Docs/Prasad_TrackA_Task_Tracker.xlsx
@@ -917,17 +917,25 @@
           <t>Track A</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Core done + tested. The node-N brain in services/event_pipeline/triggers/. Sandboxed field/op/value rule DSL (eq/ne/in/not_in/gt/gte/lt/lte/exists over dotted paths, no eval, §8). Node-N routing: idempotency guard -&gt; match active rules -&gt; deferred matches to DeferredSink (M06/A7), in-session matches to A6.reserve; approved -&gt; FireMessage on FireSink (M08/B2), suppressed -&gt; SuppressionSink (Z1/M14), no match -&gt; dropped. Contracts are messages to sinks not direct calls (§5); FireMessage (generator/models.py) carries A6's reservation_id. RedisTriggerConsumer (XREADGROUP events:in/group trigger-eval -&gt; evaluate -&gt; XACK) + parse_stream_fields; end-to-end store-&gt;relay-&gt;parse-&gt;evaluate-&gt;fire tested with no Redis. Deferred (POA/04 §11): I/J derivation workers (need A7), rule hot-reload, handoff branch (§10.3), consumer partitioning.</t>
+        </is>
+      </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>NEXT. Depends on A2, A6 (both done). Consumes the Redis stream (events:in / group trigger-eval), matches triggers, hands MatchCandidates to A6's reserve(), and emits the 'fire' decision as a Pydantic message (§5). Code against generator/fixtures.py trigger defaults until B1 ships persistence.</t>
+          <t>services/event_pipeline/triggers/{dsl,evaluator,consumer,sinks}.py, generator/models.py (FireMessage), POA/04 §11; tests/test_trigger_evaluation.py (12) — 146 total green, ruff clean. Commit 2b46310 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -997,7 +1005,7 @@
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Depends on A2, A5. make_celery() factory already stubbed in services/platform (celery added as a dep here).</t>
+          <t>NEXT. Depends on A2, A5 (both done). Consumes A5's DeferredSink items + runs the I/J derivation scans A5 deferred (uses A2 read models: has_repeated_search, last_event_at). make_celery() factory already stubbed in services/platform (celery added as a dep here).</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1505,6 +1513,33 @@
       <c r="E12" s="4" t="inlineStr">
         <is>
           <t>7a5a0f8 (PR #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Built the trigger engine — node N, the brain that ties A2, A6 and (eventually) M08 together. Kept A5 thin on purpose: matching is a small sandboxed field/op/value DSL (no eval), cap/precedence is delegated to A6, and every downstream is a message to a sink rather than a direct call (POA/18 §5) so Track B's M08 and my own A7 plug in without A5 changing. The fire decision is a shared FireMessage carrying A6's reservation_id, so the confirm/rollback loop reaches back to the cap. Added an idempotency guard so an at-least-once stream redelivery can't double-fire, and an end-to-end test that runs a real ingested event through store-&gt;relay-&gt;parse-&gt;evaluate-&gt;fire without needing Redis. Scoped POA/04 §11 honestly: the I/J derivation workers wait on A7, and the handoff branch on M07/§10.3.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>12 new tests, 146 total green; ruff clean</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>2b46310 (PR #1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: A7 done + work-log row; A8 marked next
Regenerate Docs/Prasad_TrackA_Task_Tracker.xlsx: A7 Pending Queue/Scheduler ->
in progress with detail (commit 10285b5), A8 Human Handoff marked next, Work Log
row for A7.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgpcHPiZiSoedUk6eogriY
</commit_message>
<xml_diff>
--- a/Docs/Prasad_TrackA_Task_Tracker.xlsx
+++ b/Docs/Prasad_TrackA_Task_Tracker.xlsx
@@ -995,17 +995,25 @@
           <t>Track A</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Core done + tested. services/event_pipeline/pending/: pending_engagements queue where PendingQueue.enqueue IS A5's DeferredSink (so A5's deferred matches flow straight in, no duplication). eligible_at = created + wait_period, expires_at = created + expiry; every read takes an explicit `now` so wait/eligibility/expiry are time-travel tested. expire_due sweeps overdue pending -&gt; expired (returns ids for Z2), never touching raised/raising; reconcile_stuck releases crashed `raising` rows. Login re-eval (node S): on_login under a per-customer lock fetches eligible entries, arbitrates them through A6 (multiple pending compete on PRECEDENCE, §10.3), fires the winner via FireSink + marks raised; losers/cap-suppressed stay pending for a later login. Concurrency test: 5 parallel logins raise at most once. Celery Beat wiring (beat_schedule + register_pending_tasks) with no top-level celery import. e2e A5-&gt;A7-&gt;A6 tested. Deferred (POA/06 §11): in-session merge at login, SKIP-LOCKED claim, Beat integration run.</t>
+        </is>
+      </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>NEXT. Depends on A2, A5 (both done). Consumes A5's DeferredSink items + runs the I/J derivation scans A5 deferred (uses A2 read models: has_repeated_search, last_event_at). make_celery() factory already stubbed in services/platform (celery added as a dep here).</t>
+          <t>services/event_pipeline/pending/{tables,queue,scheduler,tasks,bootstrap}.py, services/requirements.txt + pyproject (celery), POA/06 §11; tests/test_pending_queue.py (12) — 158 total green, ruff clean. Commit 10285b5 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1048,7 @@
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Depends on A5. Keep handoff code THIN around RoutingRule .match/.route/.sla dicts — B1 will likely tighten them into real models. Handoff event is a message contract, not a call (§5).</t>
+          <t>NEXT. Depends on A5 (done). Keep handoff code THIN around RoutingRule .match/.route/.sla dicts — B1 will likely tighten them into real models. Handoff event is a message contract, not a call (§5). Routing defaults already in generator/fixtures.default_routing_rules().</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1540,6 +1548,33 @@
       <c r="E13" s="4" t="inlineStr">
         <is>
           <t>2b46310 (PR #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Built the deferred branch — the pending queue + login re-evaluation. The clean win was making PendingQueue implement A5's DeferredSink, so A5's deferred matches flow straight in with no new contract, and on_login just re-arbitrates them through the SAME A6 engine — so precedence and cap behave identically whether a signal fires in-session or after a login. Kept it testable without a clock or a broker: every read takes an explicit `now` (so expiry/eligibility are time-travelled) and the Celery tasks are thin wrappers over pure methods with no top-level celery import. Wrote the two invariants the POA cares about — raised-at-most-once under concurrent logins, and expiry never touching a raised row. Answered §10.3 (pending entries compete on precedence, not FIFO).</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>12 new tests, 158 total green; ruff clean</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>10285b5 (PR #1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: A8 done + work-log row; A3 marked next (last Track A module)
Regenerate Docs/Prasad_TrackA_Task_Tracker.xlsx: A8 Human Handoff -> in progress
with detail (commit d23cef6), A3 Event Capture SDK marked next, Work Log row for A8.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgpcHPiZiSoedUk6eogriY
</commit_message>
<xml_diff>
--- a/Docs/Prasad_TrackA_Task_Tracker.xlsx
+++ b/Docs/Prasad_TrackA_Task_Tracker.xlsx
@@ -970,7 +970,7 @@
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Depends on the A4 contract, not the whole service.</t>
+          <t>NEXT — the last Track A module. Depends on the A4 contract (done), not the whole service. Client-side/server SDK that emits generator.models.Event to A4's POST /v1/events; the wire contract already exists, so this is the emit/batch/consent-gating layer.</t>
         </is>
       </c>
     </row>
@@ -1038,17 +1038,25 @@
           <t>Track A</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Core done + tested, kept THIN around RoutingRule's bare match/route/sla dicts (so B1/M13 can tighten them without reworking A8). services/event_pipeline/handoff/: HandoffRequest contract (a message, §5), first-match routing over the M13 dicts + catch_all default (reuses fixtures.default_routing_rules), context packaging (refs + human summary, no inlined PII — M15 §4), QueueAdapter seam (default wraps SupportQueueMock, §10.1 open) with per-queue retry, no-agent/after-hours -&gt; fallback queue, and dead-letter so a handoff is NEVER dropped silently. Lifecycle ledger (routed/fallback/dead_lettered -&gt; accepted -&gt; resolved) keyed by ticket_ref for M14 handoff-rate + closed-loop attribution. Cross-track: HandoffRequest in generator/models.py, reconcile with M12/B6. Deferred (POA/07 §11): concrete support-platform adapter, M12-&gt;M04 intake wiring.</t>
+        </is>
+      </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>NEXT. Depends on A5 (done). Keep handoff code THIN around RoutingRule .match/.route/.sla dicts — B1 will likely tighten them into real models. Handoff event is a message contract, not a call (§5). Routing defaults already in generator/fixtures.default_routing_rules().</t>
+          <t>services/event_pipeline/handoff/{routing,packager,adapter,manager,ledger,tables,bootstrap}.py, generator/models.py (contract), POA/07 §11; tests/test_handoff_manager.py (10) — 181 total green, ruff clean. Commit d23cef6 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1602,6 +1610,33 @@
       <c r="E15" s="4" t="inlineStr">
         <is>
           <t>89ebcf9 (PR #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Built the handoff manager — the escalation-to-human branch — on the engine Shagun's review had just hardened. Deliberately thin: routing reads RoutingRule's bare dicts directly rather than building types B1/M13 will replace, and context is packaged as refs + a summary, not inlined PII (the agent tool fetches the transcript by conversation_id). The failure handling is the substance — dispatch behind an adapter seam (the support platform is unknown, POA/07 §10.1), retry per queue, no-agent/after-hours falls to the fallback queue, and if every queue is exhausted the handoff is dead-lettered, never dropped silently (a lost escalation is a customer left hanging). Lifecycle ledger tracks routed-&gt;accepted-&gt;resolved by ticket_ref for M14. HandoffRequest is a message contract (§5). This completes A1-A8 — the whole Track A pipeline except the A3 capture SDK.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>10 new tests, 181 total green; ruff clean</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>d23cef6 (PR #1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: A3 done — Track A (A1-A8) complete
Regenerate Docs/Prasad_TrackA_Task_Tracker.xlsx: A3 Event Capture SDK -> in
progress with detail (commit b7a9320) + Work Log row. All Track A modules
(A1-A8) now landed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AgpcHPiZiSoedUk6eogriY
</commit_message>
<xml_diff>
--- a/Docs/Prasad_TrackA_Task_Tracker.xlsx
+++ b/Docs/Prasad_TrackA_Task_Tracker.xlsx
@@ -52,7 +52,7 @@
       <color rgb="001F3864"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -72,11 +72,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,10 +122,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -960,17 +952,25 @@
           <t>Track A</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Core done + tested — COMPLETES TRACK A. A Python reference/server-side capture SDK in services/event_pipeline/capture/ (the prod client is JS on the portal; §4.1 placement is open, so both sit behind the shared Event contract). CaptureClient builds schema-valid generator.models.Event for the 8 signals (detectors stamp the right payload — abandon carries the step, error the code), correlates a session (stable session_id, start_session on login), gates on analytics consent (off -&gt; dropped, nothing emitted), buffers to a capped queue, and flushes batches to A4's /v1/events:batch over stdlib urllib. A failed flush KEEPS the batch and retries -&gt; no loss under a transient outage. event_id is client-generated for idempotency; an SDK-&gt;A4 contract test proves valid events are accepted+stored and a lost-ack retry is deduped by A4. No models.py change (reuses Event). Deferred (POA/01 §12): the client-side JS SDK + browser detectors, sendBeacon flush, IndexedDB buffering — portal-team work behind the contract.</t>
+        </is>
+      </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>NEXT — the last Track A module. Depends on the A4 contract (done), not the whole service. Client-side/server SDK that emits generator.models.Event to A4's POST /v1/events; the wire contract already exists, so this is the emit/batch/consent-gating layer.</t>
+          <t>services/event_pipeline/capture/{client,buffer,transport,session}.py, POA/01 §12; tests/test_capture_sdk.py (9) — 190 total green, ruff clean. Commit b7a9320 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1637,6 +1637,33 @@
       <c r="E16" s="4" t="inlineStr">
         <is>
           <t>d23cef6 (PR #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Built the capture SDK — the front door — closing out Track A. In prod this is a client-side JS SDK (dwell/mid-flow-exit detection lives in the browser); who owns the portal embed is still open, so I shipped the Python reference/server-side path behind the same Event contract, which doubles as the QA harness that simulates each signal. The part worth testing is resilience: a flush that fails keeps the batch and retries, so a transient A4 outage loses nothing, and because event_id is client-generated, a lost-ack retry is deduped by A4 rather than double-counted — I wrote the end-to-end test for both. Consent gating drops behavioural events when analytics consent is off. With this, A1-A8 are all done: capture -&gt; ingest -&gt; store -&gt; stream -&gt; match -&gt; cap/precedence -&gt; fire -&gt; deferred -&gt; handoff.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>9 new tests, 190 total green; ruff clean</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>b7a9320 (PR #1)</t>
         </is>
       </c>
     </row>
@@ -1670,243 +1697,243 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>THE SPLIT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Prasad — Track A</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Event &amp; trigger pipeline + platform: POA 01-07, 15. Sprint 0: S1, S2, S5.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Shagun — Track B</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Conversation, config &amp; reporting: POA 08-14. Sprint 0: S3, S4, S6.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
+      <c r="A6" s="8" t="inlineStr"/>
+      <c r="B6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>SHARED FILES — announce before pushing</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>generator/models.py</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Both tracks need it. Append one bounded contiguous block; never rename or remove a field the other track uses. My Sprint 0 added optional fields/enums only — nothing renamed/removed.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>generator/pipeline.py</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Both add writers. Keep the diff to contiguous appended lines.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>tests/conftest.py</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Keep new fixtures in your own test module unless genuinely shared.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Golden prices are sacred</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Any world change must keep the 7 golden-scenario prices byte-stable — use the additive-pass pattern (see S1).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
+      <c r="A12" s="8" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>DECIDED — from my (Track A) side</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Repo layout</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>RATIFIED: services/ monorepo (platform + event_pipeline + conversation). Recorded in POA/15 §12; POA/18 §8.2 marked RESOLVED.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Git workflow</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Track A on long-lived branch track-a/event-pipeline; merge (not rebase) main at day-end; PR into main (PR #1 open); no force-push. To reconcile with Shagun's current local-only rule.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr"/>
-      <c r="B16" s="10" t="inlineStr"/>
+      <c r="A16" s="8" t="inlineStr"/>
+      <c r="B16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>OPEN — needs the client (POA/00 §7)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>LLM provider &amp; data residency</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Which model, which region, Hertz constraints.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Booking API</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>One service or several? Latency SLA? (gates A-side claim inputs / B4.)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>HS-103 surface</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>REST, websocket or embedded widget SDK?</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Support/agent queue</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Zendesk, Salesforce or in-house? (gates A8 handoff routing.)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr"/>
-      <c r="B22" s="10" t="inlineStr"/>
+      <c r="A22" s="8" t="inlineStr"/>
+      <c r="B22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>HOW TO USE THIS FILE</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>On starting a task</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Set Status to 'In progress' and fill Started.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>On finishing</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Set Status 'DONE', fill Completed, and write What I did + Files/evidence.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Every session</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Add a Work Log row — the log is what shows effort, the status is only a flag.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Regenerate</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>python build_prasad_tracker.py  (overwrites this file — edit the script, not just the sheet, if you want changes to survive)</t>
         </is>

</xml_diff>